<commit_message>
working model with "nice" output
</commit_message>
<xml_diff>
--- a/backend/models/test.xlsx
+++ b/backend/models/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alqer\Desktop\Kaizen\EcoKaizen\ecokaizen_alpha\backend\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F865859A-0682-42E0-8C17-26EC509C74AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE0CE919-830F-473E-B77F-9BA3D8F689DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="3840" windowWidth="19185" windowHeight="10785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -78,8 +78,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -364,161 +365,89 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
       <c r="F2">
+        <v>5.1639777946687904</v>
+      </c>
+      <c r="G2">
+        <v>2.5819888975751533</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>5.163977794772924</v>
+      </c>
+      <c r="G3">
+        <v>7.745966693799744</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>3.8729833464134442</v>
+      </c>
+      <c r="C4">
+        <v>6.4549722443686885</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>3.872983345830499</v>
+      </c>
+      <c r="C5">
+        <v>6.4549722408318235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>2.581988897695533</v>
+      </c>
+      <c r="E6">
+        <v>7.7459666899967425</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <v>4</v>
-      </c>
-      <c r="C4">
-        <v>6</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>3</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
       <c r="D7">
-        <v>8</v>
+        <v>7.7459666930865989</v>
       </c>
       <c r="E7">
-        <v>3</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
+        <v>2.5819888966655808</v>
       </c>
     </row>
   </sheetData>

</xml_diff>